<commit_message>
figure abbrev fxn updated
</commit_message>
<xml_diff>
--- a/Outputs/Annotation/QC.xlsx
+++ b/Outputs/Annotation/QC.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4026" uniqueCount="1631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4022" uniqueCount="1636">
   <si>
     <t>Identified Name</t>
   </si>
@@ -4933,6 +4933,21 @@
   </si>
   <si>
     <t>S-Adenosyl-L-methionine (SAM)</t>
+  </si>
+  <si>
+    <t>IEFVPTC</t>
+  </si>
+  <si>
+    <t>invasive encapsulated follicular variant of PTC</t>
+  </si>
+  <si>
+    <t>tricarboxylic acid</t>
+  </si>
+  <si>
+    <t>AA</t>
+  </si>
+  <si>
+    <t>amino acid</t>
   </si>
 </sst>
 </file>
@@ -14997,7 +15012,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0EDF12F-ACFA-854C-BF7A-D84A1BAF082E}">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.83203125" bestFit="1" customWidth="1"/>
@@ -15046,9 +15061,7 @@
       <c r="F2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="G2" s="3"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
@@ -15061,9 +15074,7 @@
         <v>1062</v>
       </c>
       <c r="D3" s="3"/>
-      <c r="E3" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
     </row>
@@ -15096,9 +15107,7 @@
         <v>63</v>
       </c>
       <c r="E5" s="3"/>
-      <c r="F5" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="F5" s="3"/>
       <c r="G5" s="3"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -15112,7 +15121,9 @@
         <v>615</v>
       </c>
       <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
+      <c r="E6" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="F6" s="3" t="s">
         <v>63</v>
       </c>
@@ -15160,9 +15171,7 @@
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
-      <c r="F9" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="F9" s="3"/>
       <c r="G9" s="3"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -15176,10 +15185,10 @@
         <v>1264</v>
       </c>
       <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>63</v>
       </c>
+      <c r="F10" s="3"/>
       <c r="G10" s="3"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -15207,9 +15216,7 @@
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
-      <c r="F12" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="F12" s="3"/>
       <c r="G12" s="3"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -15244,10 +15251,10 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>1569</v>
+        <v>1631</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1577</v>
+        <v>1632</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3" t="s">
@@ -15267,9 +15274,7 @@
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
-      <c r="F16" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="F16" s="3"/>
       <c r="G16" s="3"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -15283,8 +15288,12 @@
         <v>607</v>
       </c>
       <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
+      <c r="E17" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="G17" s="3" t="s">
         <v>63</v>
       </c>
@@ -15316,9 +15325,7 @@
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
-      <c r="F19" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="F19" s="3"/>
       <c r="G19" s="3"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -15418,13 +15425,9 @@
         <v>1579</v>
       </c>
       <c r="C25" s="3"/>
-      <c r="D25" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="D25" s="3"/>
       <c r="E25" s="3"/>
-      <c r="F25" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="F25" s="3"/>
       <c r="G25" s="3"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -15490,7 +15493,9 @@
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
+      <c r="F29" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="G29" s="3" t="s">
         <v>63</v>
       </c>
@@ -15505,9 +15510,7 @@
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
-      <c r="F30" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="F30" s="3"/>
       <c r="G30" s="3"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -15515,7 +15518,7 @@
         <v>1593</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>1603</v>
+        <v>1633</v>
       </c>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
@@ -15535,15 +15538,28 @@
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="3" t="s">
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A33" s="3" t="s">
+        <v>1634</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>1635</v>
+      </c>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G32" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G32" xr:uid="{E0EDF12F-ACFA-854C-BF7A-D84A1BAF082E}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G32">
-      <sortCondition ref="A1:A32"/>
+  <autoFilter ref="A1:G33" xr:uid="{E0EDF12F-ACFA-854C-BF7A-D84A1BAF082E}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G33">
+      <sortCondition ref="A1:A33"/>
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="C1:C1048576 A1:A1048576">

</xml_diff>